<commit_message>
More E2E artefacts from the running sweep
Twelve further files from scripts 2 and 3 of the 48-script re-run —
screenshots and generated workbooks, nothing outside e2e-screenshots/.

Committed as they land rather than in one batch at the end. The run takes
about an hour and this container has reset three times today, each time
discarding everything not pushed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/accessory-reupload-reconcile/sales-accessory.xlsx
+++ b/e2e-screenshots/accessory-reupload-reconcile/sales-accessory.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="53">
   <si>
     <t>Date</t>
   </si>
@@ -746,7 +746,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -759,38 +759,20 @@
       <c r="D2" t="s">
         <v>34</v>
       </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>35</v>
       </c>
-      <c r="F2">
+      <c r="I2">
         <v>2</v>
       </c>
-      <c r="G2">
+      <c r="J2">
         <v>3.5</v>
       </c>
-      <c r="H2">
+      <c r="K2">
         <v>8.99</v>
       </c>
-      <c r="I2" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2" t="s">
-        <v>34</v>
-      </c>
-      <c r="K2" t="s">
-        <v>34</v>
-      </c>
-      <c r="L2">
+      <c r="R2">
         <v>0</v>
-      </c>
-      <c r="M2" t="s">
-        <v>34</v>
-      </c>
-      <c r="N2" t="s">
-        <v>34</v>
-      </c>
-      <c r="O2" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>